<commit_message>
fix(i18n): synchronize and verify 100% Japanese translations with Excel master
</commit_message>
<xml_diff>
--- a/TraderRank_Translations_3Languages.xlsx
+++ b/TraderRank_Translations_3Languages.xlsx
@@ -23,7 +23,7 @@
     <t>TRADERRANK MULTI-LANGUAGE TRANSLATION MATRIX (EN / JA / ZH)</t>
   </si>
   <si>
-    <t>Generated on 2026-10-07 • Total Keys: 748 • All 3 Languages Unified for Side-by-Side Verification</t>
+    <t>Generated on 2026-10-29 • Total Keys: 748 • All 3 Languages Unified for Side-by-Side Verification</t>
   </si>
   <si>
     <t>Module / Category</t>
@@ -1220,13 +1220,13 @@
     <t>intel.doNotEnterTrade</t>
   </si>
   <si>
-    <t>⛔ DO NOT ENTER TRADE • INSUFFICIENT {targetRR} R:R</t>
-  </si>
-  <si>
-    <t>⛔ トレードエントリー禁止 • 目標 {targetRR} R:R 未達</t>
-  </si>
-  <si>
-    <t>⛔ 禁止入场交易 • 目标 {targetRR} R:R 盈亏比不足</t>
+    <t>[HOLD] DO NOT ENTER TRADE • INSUFFICIENT {targetRR} R:R</t>
+  </si>
+  <si>
+    <t>[HOLD] トレードエントリー禁止 • 目標 {targetRR} R:R 未達</t>
+  </si>
+  <si>
+    <t>[HOLD] 暂缓入场交易 • 目标 {targetRR} R:R 盈亏比不足</t>
   </si>
   <si>
     <t>intel.rrTargetsLabel</t>
@@ -1280,13 +1280,13 @@
     <t>intel.switchScan</t>
   </si>
   <si>
-    <t>⚡ Switch &amp; Scan</t>
-  </si>
-  <si>
-    <t>⚡ 切り替えてスキャン</t>
-  </si>
-  <si>
-    <t>⚡ 切换并即时扫描</t>
+    <t>Switch &amp; Scan</t>
+  </si>
+  <si>
+    <t>切り替えてスキャン</t>
+  </si>
+  <si>
+    <t>切换并即时扫描</t>
   </si>
   <si>
     <t>intel.confluenceScore</t>
@@ -2015,13 +2015,13 @@
     <t>chart.aiAnalysisBtn</t>
   </si>
   <si>
-    <t>⚡ AI Smart Analysis</t>
-  </si>
-  <si>
-    <t>⚡ AIスマート分析</t>
-  </si>
-  <si>
-    <t>⚡ AI智能深度剖析</t>
+    <t>AI Smart Analysis</t>
+  </si>
+  <si>
+    <t>AIスマート分析</t>
+  </si>
+  <si>
+    <t>AI智能深度剖析</t>
   </si>
   <si>
     <t>chart.lastPrice</t>
@@ -2123,13 +2123,13 @@
     <t>chart.demandSupplyLabel</t>
   </si>
   <si>
-    <t>⚡ Demand &amp; Supply Zones</t>
-  </si>
-  <si>
-    <t>⚡ デマンド &amp; サプライゾーン</t>
-  </si>
-  <si>
-    <t>⚡ 供需区间 (Demand &amp; Supply)</t>
+    <t>Demand &amp; Supply Zones</t>
+  </si>
+  <si>
+    <t>デマンド &amp; サプライゾーン</t>
+  </si>
+  <si>
+    <t>供需区间 (Demand &amp; Supply)</t>
   </si>
   <si>
     <t>chart.demandSupplyDesc</t>
@@ -2147,13 +2147,13 @@
     <t>chart.bosLabel</t>
   </si>
   <si>
-    <t>📊 Break of Structure (BOS / CHoCH)</t>
-  </si>
-  <si>
-    <t>📊 構造ブレイク (BOS / CHoCH)</t>
-  </si>
-  <si>
-    <t>📊 结构突破 (BOS / CHoCH)</t>
+    <t>Break of Structure (BOS / CHoCH)</t>
+  </si>
+  <si>
+    <t>構造ブレイク (BOS / CHoCH)</t>
+  </si>
+  <si>
+    <t>结构突破 (BOS / CHoCH)</t>
   </si>
   <si>
     <t>chart.bosDesc</t>
@@ -2318,37 +2318,37 @@
     <t>chart.closeSubPanel</t>
   </si>
   <si>
-    <t>✕ Close Sub-Panel</t>
-  </si>
-  <si>
-    <t>✕ サブパネルを閉じる</t>
-  </si>
-  <si>
-    <t>✕ 关闭副图面板</t>
+    <t>Close Sub-Panel</t>
+  </si>
+  <si>
+    <t>サブパネルを閉じる</t>
+  </si>
+  <si>
+    <t>关闭副图面板</t>
   </si>
   <si>
     <t>chart.liveStreamActive</t>
   </si>
   <si>
-    <t>AllTick Live Stream: ForexFactory Red Folder Calendar &amp; AI Engine Active</t>
-  </si>
-  <si>
-    <t>AllTick ライブ配信: ForexFactory 赤フォルダ &amp; AIエンジン稼働中</t>
-  </si>
-  <si>
-    <t>AllTick 实时流: ForexFactory 财经日历与 AI 引擎运作中</t>
+    <t>MetaApi Broker Stream: Live Forex &amp; Gold Feed Active</t>
+  </si>
+  <si>
+    <t>MetaApi ブローカーストリーム: ライブ為替・ゴールド配信中</t>
+  </si>
+  <si>
+    <t>MetaApi 经纪商数据流: 实时外汇与黄金行情已连接</t>
   </si>
   <si>
     <t>chart.tokenTrial</t>
   </si>
   <si>
-    <t>Token: 4554c41c...-c-app (7-Day Trial)</t>
-  </si>
-  <si>
-    <t>トークン: 4554c41c...-c-app (7日間トライアル)</t>
-  </si>
-  <si>
-    <t>授权令牌: 4554c41c...-c-app (7天试用)</t>
+    <t>MetaApi Cloud Broker Ledger (Live)</t>
+  </si>
+  <si>
+    <t>MetaApi クラウドブローカー台帳 (ライブ)</t>
+  </si>
+  <si>
+    <t>MetaApi 云经纪商交易账本 (实时)</t>
   </si>
   <si>
     <t>chart.overlayIndicators</t>
@@ -2873,13 +2873,13 @@
     <t>subscription.congratsTitle</t>
   </si>
   <si>
-    <t>🎉 Welcome to TraderRank Pro!</t>
-  </si>
-  <si>
-    <t>🎉 TraderRank Pro へようこそ！</t>
-  </si>
-  <si>
-    <t>🎉 欢迎加入 TraderRank Pro！</t>
+    <t>Welcome to TraderRank Pro</t>
+  </si>
+  <si>
+    <t>TraderRank Pro へようこそ</t>
+  </si>
+  <si>
+    <t>欢迎加入 TraderRank Pro</t>
   </si>
   <si>
     <t>subscription.congratsSubtitle</t>
@@ -3800,13 +3800,13 @@
     <t>connector.preflightPassed</t>
   </si>
   <si>
-    <t>✓ Preflight Passed — Read-Only Verified</t>
-  </si>
-  <si>
-    <t>✓ 事前テスト合格 — 閲覧専用確認済み</t>
-  </si>
-  <si>
-    <t>✓ 预检通过 — 只读权限验真成功</t>
+    <t>Preflight Passed — Read-Only Verified</t>
+  </si>
+  <si>
+    <t>事前テスト合格 — 閲覧専用確認済み</t>
+  </si>
+  <si>
+    <t>预检通过 — 只读权限验真成功</t>
   </si>
   <si>
     <t>connector.stepBroker</t>
@@ -4772,13 +4772,13 @@
     <t>rewards.streakActive</t>
   </si>
   <si>
-    <t>🔥 4-Day Active Streak!</t>
-  </si>
-  <si>
-    <t>🔥 4日連続アクティブ継続中！</t>
-  </si>
-  <si>
-    <t>🔥 已连续保持 4 天活跃！</t>
+    <t>4-Day Active Streak</t>
+  </si>
+  <si>
+    <t>4日連続アクティブ継続中</t>
+  </si>
+  <si>
+    <t>已连续保持 4 天活跃</t>
   </si>
   <si>
     <t>rewards.claimBtn</t>
@@ -5996,49 +5996,49 @@
     <t>community.cheersBullish</t>
   </si>
   <si>
-    <t>Bullish 🐂</t>
-  </si>
-  <si>
-    <t>強気 🐂</t>
-  </si>
-  <si>
-    <t>看涨 🐂</t>
+    <t>Bullish [BULL]</t>
+  </si>
+  <si>
+    <t>強気 [BULL]</t>
+  </si>
+  <si>
+    <t>看涨 [BULL]</t>
   </si>
   <si>
     <t>community.cheersRocket</t>
   </si>
   <si>
-    <t>Rocket 🚀</t>
-  </si>
-  <si>
-    <t>急上昇 🚀</t>
-  </si>
-  <si>
-    <t>起飞 🚀</t>
+    <t>Breakout [EXP]</t>
+  </si>
+  <si>
+    <t>急上昇 [EXP]</t>
+  </si>
+  <si>
+    <t>强势突破 [EXP]</t>
   </si>
   <si>
     <t>community.cheersKing</t>
   </si>
   <si>
-    <t>Alpha 👑</t>
-  </si>
-  <si>
-    <t>覇者 👑</t>
-  </si>
-  <si>
-    <t>霸气 👑</t>
+    <t>Alpha [LEAD]</t>
+  </si>
+  <si>
+    <t>覇者 [LEAD]</t>
+  </si>
+  <si>
+    <t>领航 [LEAD]</t>
   </si>
   <si>
     <t>community.cheersShield</t>
   </si>
   <si>
-    <t>Risk Guard 🛡️</t>
-  </si>
-  <si>
-    <t>鉄壁の防衛 🛡️</t>
-  </si>
-  <si>
-    <t>稳如泰山 🛡️</t>
+    <t>Risk Guard [DEF]</t>
+  </si>
+  <si>
+    <t>鉄壁の防衛 [DEF]</t>
+  </si>
+  <si>
+    <t>防守大师 [DEF]</t>
   </si>
   <si>
     <t>community.justNow</t>
@@ -7010,13 +7010,13 @@
     <t>aiModal.plottedOnChartBtn</t>
   </si>
   <si>
-    <t>✓ AI Levels Plotted on Chart</t>
-  </si>
-  <si>
-    <t>✓ AI水準を描画中</t>
-  </si>
-  <si>
-    <t>✓ 已在图表上标绘 AI 关键位</t>
+    <t>AI Levels Plotted on Chart</t>
+  </si>
+  <si>
+    <t>AI水準を描画中</t>
+  </si>
+  <si>
+    <t>已在图表上标绘 AI 关键位</t>
   </si>
   <si>
     <t>aiModal.multiTfStructureBreakdown</t>
@@ -13672,7 +13672,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="195" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="8" t="s">
         <v>599</v>
       </c>
@@ -31273,7 +31273,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="24" t="s">
         <v>399</v>
       </c>

</xml_diff>

<commit_message>
fix(i18n): fix Japanese word wrapping, unlock terminology and button text formatting
</commit_message>
<xml_diff>
--- a/TraderRank_Translations_3Languages.xlsx
+++ b/TraderRank_Translations_3Languages.xlsx
@@ -191,13 +191,13 @@
     <t>nav.connectAccount</t>
   </si>
   <si>
-    <t>+ Connect Broker</t>
-  </si>
-  <si>
-    <t>+ 口座を連携</t>
-  </si>
-  <si>
-    <t>+ 绑定经纪商</t>
+    <t>Connect Broker</t>
+  </si>
+  <si>
+    <t>口座を連携</t>
+  </si>
+  <si>
+    <t>绑定经纪商</t>
   </si>
   <si>
     <t>nav.proLeague</t>
@@ -230,7 +230,7 @@
     <t>Unlock Pro ($9/mo)</t>
   </si>
   <si>
-    <t>Pro を解除 ($9/月)</t>
+    <t>Pro をアンロック ($9/月)</t>
   </si>
   <si>
     <t>解锁 Pro 权限 ($9/月)</t>
@@ -812,7 +812,7 @@
     <t>PRO UNLOCKED ($9/mo)</t>
   </si>
   <si>
-    <t>PRO 解除済み ($9/月)</t>
+    <t>PRO アンロック済み ($9/月)</t>
   </si>
   <si>
     <t>PRO 权限已解锁 ($9/月)</t>
@@ -824,7 +824,7 @@
     <t>Unlock Pro for $9/Month</t>
   </si>
   <si>
-    <t>月額 $9 で Pro を解除</t>
+    <t>月額 $9 で Pro をアンロック</t>
   </si>
   <si>
     <t>以 $9/月 解锁 Pro 权限</t>
@@ -1454,7 +1454,7 @@
     <t>Unlock Custom Strategic Timeframe Generator</t>
   </si>
   <si>
-    <t>カスタム時間軸戦略ジェネレーターを解除</t>
+    <t>カスタム時間軸戦略ジェネレーターをアンロック</t>
   </si>
   <si>
     <t>解锁定制时间周期策略生成器</t>
@@ -1478,7 +1478,7 @@
     <t>Unlock for $9 / Month</t>
   </si>
   <si>
-    <t>月額 $9 で解除する</t>
+    <t>月額 $9 でアンロックする</t>
   </si>
   <si>
     <t>以 $9/月 立即解锁</t>

</xml_diff>